<commit_message>
Update Transmitter_v3 mit powerManager zum Laden
</commit_message>
<xml_diff>
--- a/doc/ESP32_Pinning_Transmitter.xlsx
+++ b/doc/ESP32_Pinning_Transmitter.xlsx
@@ -1,23 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1a2760580a95eec9/_Projekte/ewinch_rc_jm/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{EB437FFB-F53C-5D44-8E84-1BC8140A599F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D72EE9A9-96B4-EC42-9E05-48AF90E16AAC}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="13_ncr:1_{EB437FFB-F53C-5D44-8E84-1BC8140A599F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6382027-61A1-A34D-AE9C-7439FDCF42E5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" activeTab="2" xr2:uid="{A12475C3-A2AC-8B4F-A382-743418FD4D1E}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" activeTab="3" xr2:uid="{A12475C3-A2AC-8B4F-A382-743418FD4D1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Transmitter" sheetId="1" r:id="rId1"/>
     <sheet name="Transceiver" sheetId="3" r:id="rId2"/>
-    <sheet name="Tabelle1" sheetId="4" r:id="rId3"/>
+    <sheet name="Receiver_HeltecV3" sheetId="4" r:id="rId3"/>
+    <sheet name="Receiver_HeltecV2" sheetId="5" r:id="rId4"/>
+    <sheet name="Sender_HeltecV2" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">Receiver_HeltecV2!$A$1:$O$27</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="54">
   <si>
     <t>kein PU</t>
   </si>
@@ -146,6 +151,60 @@
   </si>
   <si>
     <t>LED_GN_OUT</t>
+  </si>
+  <si>
+    <t>Supply</t>
+  </si>
+  <si>
+    <t>Rx</t>
+  </si>
+  <si>
+    <t>Tx</t>
+  </si>
+  <si>
+    <t>Lora</t>
+  </si>
+  <si>
+    <t>OLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- </t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>PWM_out</t>
+  </si>
+  <si>
+    <t>Cutter_out</t>
+  </si>
+  <si>
+    <t>Warnleuchte</t>
+  </si>
+  <si>
+    <t>Lüfter</t>
+  </si>
+  <si>
+    <t>Analog In Windrichtung</t>
+  </si>
+  <si>
+    <t>Lora opt.</t>
+  </si>
+  <si>
+    <t>RotaryPush</t>
+  </si>
+  <si>
+    <t>Vbatt</t>
+  </si>
+  <si>
+    <t>Int Pin für Ubatt</t>
+  </si>
+  <si>
+    <t>BTN Up</t>
+  </si>
+  <si>
+    <t>BTN Down</t>
   </si>
 </sst>
 </file>
@@ -206,11 +265,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -398,8 +458,102 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>508000</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>140369</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>987595</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>163495</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5CC449E-C617-E0ED-7214-C75AF4187AAA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2165684" y="741948"/>
+          <a:ext cx="8768016" cy="4635231"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>508000</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>140369</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>987595</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>163495</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B66017F-28CE-3F4C-9F4E-30901C8D29A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2159000" y="749969"/>
+          <a:ext cx="8734595" cy="4696726"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1006,4 +1160,252 @@
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E73F5CAB-9783-D340-9CF8-91FA1DBB2787}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B8:N25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="13" max="13" width="13.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B14" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="N15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="N16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="N17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="N21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="N22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="N24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10D4708A-DD57-DE48-B87A-C7EDC311E635}">
+  <dimension ref="B8:N25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="13" max="13" width="13.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B14" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="N15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="N17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="N21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="N22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>